<commit_message>
finishing 30% from users dashboard
</commit_message>
<xml_diff>
--- a/stages.xlsx
+++ b/stages.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28014"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{178C9A55-EDAD-4D92-BCC8-02F6774A6E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>id</t>
   </si>
@@ -46,12 +45,21 @@
   </si>
   <si>
     <t>مرحلة خاصة</t>
+  </si>
+  <si>
+    <t>leader_username</t>
+  </si>
+  <si>
+    <t>S27-0001</t>
+  </si>
+  <si>
+    <t>farid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -362,23 +370,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.5546875" customWidth="1"/>
-    <col min="3" max="3" width="7.33203125" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -386,23 +397,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -410,7 +427,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -420,5 +437,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cleaning up project - fixing families and stages with users bugs
</commit_message>
<xml_diff>
--- a/stages.xlsx
+++ b/stages.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28014"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\marmina\api\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577FC8A7-8154-4B58-9B9B-ADC90AA41964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336"/>
+    <workbookView xWindow="-20610" yWindow="2610" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -50,16 +51,16 @@
     <t>leader_username</t>
   </si>
   <si>
-    <t>S27-0001</t>
-  </si>
-  <si>
-    <t>farid</t>
+    <t>S30-0002</t>
+  </si>
+  <si>
+    <t>S30-0008</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -370,7 +371,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>